<commit_message>
Melhorias na pagina Conferidor e loader
</commit_message>
<xml_diff>
--- a/datasets/Jogos_Realizados.xlsx
+++ b/datasets/Jogos_Realizados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c202df0411a927e/Documentos/Python/Lotofacil/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{3777E336-E7E6-422B-B02D-717A1FC825FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52B53022-D828-437F-9C3C-AE7BC6F47299}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="8_{3777E336-E7E6-422B-B02D-717A1FC825FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE5653E7-3D3D-4EC5-A9DA-AA7EE8543C36}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B259EE94-4149-4BBF-83A3-7FF40C056672}"/>
   </bookViews>
@@ -506,21 +506,12 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="3" width="15.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="9.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="23" width="9.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9.5703125" style="2" customWidth="1"/>
+    <col min="4" max="23" width="8.140625" style="2" customWidth="1"/>
     <col min="24" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,7 +587,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>3692</v>
+        <v>3603</v>
       </c>
       <c r="C2" s="3">
         <v>3702</v>
@@ -611,43 +602,47 @@
         <v>3</v>
       </c>
       <c r="G2" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H2" s="3">
+        <v>6</v>
+      </c>
+      <c r="I2" s="3">
         <v>7</v>
       </c>
-      <c r="I2" s="3">
-        <v>8</v>
-      </c>
       <c r="J2" s="3">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K2" s="3">
+        <v>12</v>
+      </c>
+      <c r="L2" s="3">
         <v>13</v>
       </c>
-      <c r="L2" s="3">
-        <v>14</v>
-      </c>
       <c r="M2" s="3">
+        <v>15</v>
+      </c>
+      <c r="N2" s="3">
         <v>17</v>
       </c>
-      <c r="N2" s="3">
+      <c r="O2" s="3">
         <v>18</v>
       </c>
-      <c r="O2" s="3">
+      <c r="P2" s="3">
         <v>19</v>
       </c>
-      <c r="P2" s="3">
+      <c r="Q2" s="3">
+        <v>21</v>
+      </c>
+      <c r="R2" s="3">
         <v>23</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="S2" s="3">
         <v>24</v>
       </c>
-      <c r="R2" s="3">
+      <c r="T2" s="3">
         <v>25</v>
       </c>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
@@ -658,7 +653,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3">
-        <v>3692</v>
+        <v>3603</v>
       </c>
       <c r="C3" s="3">
         <v>3702</v>
@@ -679,37 +674,41 @@
         <v>7</v>
       </c>
       <c r="I3" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J3" s="3">
+        <v>10</v>
+      </c>
+      <c r="K3" s="3">
         <v>11</v>
       </c>
-      <c r="K3" s="3">
+      <c r="L3" s="3">
         <v>12</v>
       </c>
-      <c r="L3" s="3">
-        <v>15</v>
-      </c>
       <c r="M3" s="3">
+        <v>14</v>
+      </c>
+      <c r="N3" s="3">
         <v>17</v>
       </c>
-      <c r="N3" s="3">
+      <c r="O3" s="3">
         <v>19</v>
       </c>
-      <c r="O3" s="3">
+      <c r="P3" s="3">
         <v>21</v>
       </c>
-      <c r="P3" s="3">
+      <c r="Q3" s="3">
+        <v>22</v>
+      </c>
+      <c r="R3" s="3">
         <v>23</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="S3" s="3">
         <v>24</v>
       </c>
-      <c r="R3" s="3">
+      <c r="T3" s="3">
         <v>25</v>
       </c>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -720,49 +719,49 @@
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>3692</v>
+        <v>3603</v>
       </c>
       <c r="C4" s="3">
         <v>3702</v>
       </c>
       <c r="D4" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="3">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3">
+        <v>4</v>
+      </c>
+      <c r="G4" s="3">
         <v>5</v>
       </c>
-      <c r="F4" s="3">
-        <v>6</v>
-      </c>
-      <c r="G4" s="3">
-        <v>8</v>
-      </c>
       <c r="H4" s="3">
+        <v>7</v>
+      </c>
+      <c r="I4" s="3">
         <v>9</v>
       </c>
-      <c r="I4" s="3">
-        <v>10</v>
-      </c>
       <c r="J4" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K4" s="3">
+        <v>13</v>
+      </c>
+      <c r="L4" s="3">
         <v>14</v>
       </c>
-      <c r="L4" s="3">
-        <v>16</v>
-      </c>
       <c r="M4" s="3">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="N4" s="3">
+        <v>17</v>
+      </c>
+      <c r="O4" s="3">
         <v>19</v>
       </c>
-      <c r="O4" s="3">
+      <c r="P4" s="3">
         <v>21</v>
-      </c>
-      <c r="P4" s="3">
-        <v>22</v>
       </c>
       <c r="Q4" s="3">
         <v>23</v>
@@ -782,16 +781,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="3">
-        <v>3692</v>
+        <v>3603</v>
       </c>
       <c r="C5" s="3">
         <v>3702</v>
       </c>
       <c r="D5" s="3">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3">
         <v>3</v>
-      </c>
-      <c r="E5" s="3">
-        <v>5</v>
       </c>
       <c r="F5" s="3">
         <v>7</v>
@@ -803,10 +802,10 @@
         <v>9</v>
       </c>
       <c r="I5" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J5" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K5" s="3">
         <v>14</v>
@@ -815,16 +814,16 @@
         <v>15</v>
       </c>
       <c r="M5" s="3">
+        <v>16</v>
+      </c>
+      <c r="N5" s="3">
         <v>17</v>
       </c>
-      <c r="N5" s="3">
+      <c r="O5" s="3">
         <v>18</v>
       </c>
-      <c r="O5" s="3">
+      <c r="P5" s="3">
         <v>19</v>
-      </c>
-      <c r="P5" s="3">
-        <v>20</v>
       </c>
       <c r="Q5" s="3">
         <v>21</v>
@@ -848,31 +847,31 @@
         <v>5</v>
       </c>
       <c r="B6" s="3">
-        <v>3692</v>
+        <v>3603</v>
       </c>
       <c r="C6" s="3">
         <v>3702</v>
       </c>
       <c r="D6" s="3">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3">
         <v>4</v>
       </c>
-      <c r="E6" s="3">
-        <v>5</v>
-      </c>
       <c r="F6" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G6" s="3">
         <v>9</v>
       </c>
       <c r="H6" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I6" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J6" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K6" s="3">
         <v>14</v>
@@ -906,63 +905,25 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3">
-        <v>3692</v>
-      </c>
-      <c r="C7" s="3">
-        <v>3702</v>
-      </c>
-      <c r="D7" s="3">
-        <v>4</v>
-      </c>
-      <c r="E7" s="3">
-        <v>6</v>
-      </c>
-      <c r="F7" s="3">
-        <v>7</v>
-      </c>
-      <c r="G7" s="3">
-        <v>8</v>
-      </c>
-      <c r="H7" s="3">
-        <v>9</v>
-      </c>
-      <c r="I7" s="3">
-        <v>10</v>
-      </c>
-      <c r="J7" s="3">
-        <v>13</v>
-      </c>
-      <c r="K7" s="3">
-        <v>14</v>
-      </c>
-      <c r="L7" s="3">
-        <v>15</v>
-      </c>
-      <c r="M7" s="3">
-        <v>17</v>
-      </c>
-      <c r="N7" s="3">
-        <v>19</v>
-      </c>
-      <c r="O7" s="3">
-        <v>20</v>
-      </c>
-      <c r="P7" s="3">
-        <v>22</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>23</v>
-      </c>
-      <c r="R7" s="3">
-        <v>24</v>
-      </c>
-      <c r="S7" s="3">
-        <v>25</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
@@ -970,60 +931,24 @@
       <c r="X7" s="3"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3">
-        <v>3692</v>
-      </c>
-      <c r="C8" s="3">
-        <v>3702</v>
-      </c>
-      <c r="D8" s="3">
-        <v>3</v>
-      </c>
-      <c r="E8" s="3">
-        <v>5</v>
-      </c>
-      <c r="F8" s="3">
-        <v>8</v>
-      </c>
-      <c r="G8" s="3">
-        <v>9</v>
-      </c>
-      <c r="H8" s="3">
-        <v>11</v>
-      </c>
-      <c r="I8" s="3">
-        <v>12</v>
-      </c>
-      <c r="J8" s="3">
-        <v>13</v>
-      </c>
-      <c r="K8" s="3">
-        <v>15</v>
-      </c>
-      <c r="L8" s="3">
-        <v>17</v>
-      </c>
-      <c r="M8" s="3">
-        <v>18</v>
-      </c>
-      <c r="N8" s="3">
-        <v>19</v>
-      </c>
-      <c r="O8" s="3">
-        <v>21</v>
-      </c>
-      <c r="P8" s="3">
-        <v>23</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>24</v>
-      </c>
-      <c r="R8" s="3">
-        <v>25</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
@@ -1032,60 +957,24 @@
       <c r="X8" s="3"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3">
-        <v>3692</v>
-      </c>
-      <c r="C9" s="3">
-        <v>3702</v>
-      </c>
-      <c r="D9" s="3">
-        <v>3</v>
-      </c>
-      <c r="E9" s="3">
-        <v>6</v>
-      </c>
-      <c r="F9" s="3">
-        <v>7</v>
-      </c>
-      <c r="G9" s="3">
-        <v>8</v>
-      </c>
-      <c r="H9" s="3">
-        <v>9</v>
-      </c>
-      <c r="I9" s="3">
-        <v>11</v>
-      </c>
-      <c r="J9" s="3">
-        <v>13</v>
-      </c>
-      <c r="K9" s="3">
-        <v>14</v>
-      </c>
-      <c r="L9" s="3">
-        <v>15</v>
-      </c>
-      <c r="M9" s="3">
-        <v>17</v>
-      </c>
-      <c r="N9" s="3">
-        <v>18</v>
-      </c>
-      <c r="O9" s="3">
-        <v>20</v>
-      </c>
-      <c r="P9" s="3">
-        <v>21</v>
-      </c>
-      <c r="Q9" s="3">
-        <v>22</v>
-      </c>
-      <c r="R9" s="3">
-        <v>23</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
@@ -1094,60 +983,24 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3">
-        <v>3692</v>
-      </c>
-      <c r="C10" s="3">
-        <v>3702</v>
-      </c>
-      <c r="D10" s="3">
-        <v>2</v>
-      </c>
-      <c r="E10" s="3">
-        <v>4</v>
-      </c>
-      <c r="F10" s="3">
-        <v>5</v>
-      </c>
-      <c r="G10" s="3">
-        <v>7</v>
-      </c>
-      <c r="H10" s="3">
-        <v>8</v>
-      </c>
-      <c r="I10" s="3">
-        <v>10</v>
-      </c>
-      <c r="J10" s="3">
-        <v>12</v>
-      </c>
-      <c r="K10" s="3">
-        <v>13</v>
-      </c>
-      <c r="L10" s="3">
-        <v>14</v>
-      </c>
-      <c r="M10" s="3">
-        <v>15</v>
-      </c>
-      <c r="N10" s="3">
-        <v>18</v>
-      </c>
-      <c r="O10" s="3">
-        <v>19</v>
-      </c>
-      <c r="P10" s="3">
-        <v>22</v>
-      </c>
-      <c r="Q10" s="3">
-        <v>23</v>
-      </c>
-      <c r="R10" s="3">
-        <v>25</v>
-      </c>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -1156,60 +1009,24 @@
       <c r="X10" s="3"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3">
-        <v>3692</v>
-      </c>
-      <c r="C11" s="3">
-        <v>3702</v>
-      </c>
-      <c r="D11" s="3">
-        <v>4</v>
-      </c>
-      <c r="E11" s="3">
-        <v>5</v>
-      </c>
-      <c r="F11" s="3">
-        <v>6</v>
-      </c>
-      <c r="G11" s="3">
-        <v>8</v>
-      </c>
-      <c r="H11" s="3">
-        <v>10</v>
-      </c>
-      <c r="I11" s="3">
-        <v>12</v>
-      </c>
-      <c r="J11" s="3">
-        <v>13</v>
-      </c>
-      <c r="K11" s="3">
-        <v>15</v>
-      </c>
-      <c r="L11" s="3">
-        <v>16</v>
-      </c>
-      <c r="M11" s="3">
-        <v>18</v>
-      </c>
-      <c r="N11" s="3">
-        <v>19</v>
-      </c>
-      <c r="O11" s="3">
-        <v>21</v>
-      </c>
-      <c r="P11" s="3">
-        <v>23</v>
-      </c>
-      <c r="Q11" s="3">
-        <v>24</v>
-      </c>
-      <c r="R11" s="3">
-        <v>25</v>
-      </c>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>

</xml_diff>